<commit_message>
fix up traders + manual
</commit_message>
<xml_diff>
--- a/Manual Trading/Day 3/Manual Trading.xlsx
+++ b/Manual Trading/Day 3/Manual Trading.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/92c4f7ffed9c6980/Python/IntaraTradingAlgorithm/Manual Trading/Day 3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DA082EFF-C414-4551-A8BC-B89349E5E691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="77" documentId="8_{DA082EFF-C414-4551-A8BC-B89349E5E691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{59D46149-96A7-45F5-9B1A-96C20DEA7855}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{69BC4B49-F889-447C-BB1B-4A95B93F97BC}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>prices</t>
   </si>
@@ -81,6 +81,9 @@
   </si>
   <si>
     <t>profit</t>
+  </si>
+  <si>
+    <t>as percentage of max</t>
   </si>
 </sst>
 </file>
@@ -143,6 +146,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -462,7 +469,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E73CE11-7FF4-4924-A982-F61C58722206}">
-  <dimension ref="B1:N59"/>
+  <dimension ref="B1:N62"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="19.26953125" customWidth="1"/>
@@ -487,7 +494,7 @@
         <v>11</v>
       </c>
       <c r="C2">
-        <v>850</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="2:13" x14ac:dyDescent="0.35">
@@ -495,7 +502,7 @@
         <v>1</v>
       </c>
       <c r="C3">
-        <v>750</v>
+        <v>761</v>
       </c>
       <c r="D3" t="s">
         <v>3</v>
@@ -506,7 +513,7 @@
         <v>2</v>
       </c>
       <c r="C4">
-        <v>800</v>
+        <v>861</v>
       </c>
       <c r="D4" t="s">
         <v>4</v>
@@ -543,16 +550,16 @@
         <v>670</v>
       </c>
       <c r="G8" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" ref="G8:G39" si="0">1/COUNT($F$8:$F$58)</f>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H8" t="b">
-        <f>$C$3&gt;F8</f>
+        <f t="shared" ref="H8:H39" si="1">$C$3&gt;F8</f>
         <v>1</v>
       </c>
       <c r="I8">
         <f>($C$1-$C$3)*H8</f>
-        <v>170</v>
+        <v>159</v>
       </c>
       <c r="J8" t="b">
         <f>IF(H8, FALSE, $C$4&gt;F8)</f>
@@ -563,8 +570,8 @@
         <v>0</v>
       </c>
       <c r="L8">
-        <f>IF(AND(J8,$C$4&lt;=$C$2),(($C$1-$C$2)/($C$1-$C$4))^3,0)</f>
-        <v>0</v>
+        <f t="shared" ref="L8:L24" si="2">IF(AND(J8,$C$4&lt;=$C$2),(($C$1-$C$2)/($C$1-$C$4))^3,1)</f>
+        <v>1</v>
       </c>
       <c r="M8">
         <f>K8*L8</f>
@@ -576,31 +583,31 @@
         <v>675</v>
       </c>
       <c r="G9" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="0"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H9" t="b">
-        <f>$C$3&gt;F9</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="I9">
-        <f t="shared" ref="I9:I58" si="0">($C$1-$C$3)*H9</f>
-        <v>170</v>
+        <f t="shared" ref="I9:I58" si="3">($C$1-$C$3)*H9</f>
+        <v>159</v>
       </c>
       <c r="J9" t="b">
-        <f t="shared" ref="J9:J58" si="1">IF(H9, FALSE, $C$4&gt;F9)</f>
+        <f t="shared" ref="J9:J58" si="4">IF(H9, FALSE, $C$4&gt;F9)</f>
         <v>0</v>
       </c>
       <c r="K9">
-        <f t="shared" ref="K9:K58" si="2">J9*($C$1-$C$4)</f>
+        <f t="shared" ref="K9:K58" si="5">J9*($C$1-$C$4)</f>
         <v>0</v>
       </c>
       <c r="L9">
-        <f t="shared" ref="L9:L58" si="3">IF(AND(J9,$C$4&lt;=$C$2),(($C$1-$C$2)/($C$1-$C$4))^3,0)</f>
-        <v>0</v>
+        <f t="shared" si="2"/>
+        <v>1</v>
       </c>
       <c r="M9">
-        <f t="shared" ref="M9:M58" si="4">K9*L9</f>
+        <f t="shared" ref="M9:M58" si="6">K9*L9</f>
         <v>0</v>
       </c>
     </row>
@@ -609,31 +616,31 @@
         <v>680</v>
       </c>
       <c r="G10" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="0"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H10" t="b">
-        <f>$C$3&gt;F10</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="I10">
-        <f t="shared" si="0"/>
-        <v>170</v>
+        <f t="shared" si="3"/>
+        <v>159</v>
       </c>
       <c r="J10" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="K10">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="L10">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="L10">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -642,31 +649,31 @@
         <v>685</v>
       </c>
       <c r="G11" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="0"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H11" t="b">
-        <f>$C$3&gt;F11</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="I11">
-        <f t="shared" si="0"/>
-        <v>170</v>
+        <f t="shared" si="3"/>
+        <v>159</v>
       </c>
       <c r="J11" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="K11">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="L11">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="L11">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M11">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -675,31 +682,31 @@
         <v>690</v>
       </c>
       <c r="G12" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="0"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H12" t="b">
-        <f>$C$3&gt;F12</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="I12">
-        <f t="shared" si="0"/>
-        <v>170</v>
+        <f t="shared" si="3"/>
+        <v>159</v>
       </c>
       <c r="J12" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="K12">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="L12">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="L12">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M12">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -708,31 +715,31 @@
         <v>695</v>
       </c>
       <c r="G13" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="0"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H13" t="b">
-        <f>$C$3&gt;F13</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="I13">
-        <f t="shared" si="0"/>
-        <v>170</v>
+        <f t="shared" si="3"/>
+        <v>159</v>
       </c>
       <c r="J13" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="K13">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="L13">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="L13">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M13">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -741,31 +748,31 @@
         <v>700</v>
       </c>
       <c r="G14" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="0"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H14" t="b">
-        <f>$C$3&gt;F14</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="I14">
-        <f t="shared" si="0"/>
-        <v>170</v>
+        <f t="shared" si="3"/>
+        <v>159</v>
       </c>
       <c r="J14" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="K14">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="L14">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="L14">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -774,31 +781,31 @@
         <v>705</v>
       </c>
       <c r="G15" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="0"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H15" t="b">
-        <f>$C$3&gt;F15</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="I15">
-        <f t="shared" si="0"/>
-        <v>170</v>
+        <f t="shared" si="3"/>
+        <v>159</v>
       </c>
       <c r="J15" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="K15">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="L15">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="L15">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M15">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -807,31 +814,31 @@
         <v>710</v>
       </c>
       <c r="G16" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="0"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H16" t="b">
-        <f>$C$3&gt;F16</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="I16">
-        <f t="shared" si="0"/>
-        <v>170</v>
+        <f t="shared" si="3"/>
+        <v>159</v>
       </c>
       <c r="J16" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="K16">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="L16">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="L16">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M16">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -840,31 +847,31 @@
         <v>715</v>
       </c>
       <c r="G17" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="0"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H17" t="b">
-        <f>$C$3&gt;F17</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="I17">
-        <f t="shared" si="0"/>
-        <v>170</v>
+        <f t="shared" si="3"/>
+        <v>159</v>
       </c>
       <c r="J17" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="K17">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="L17">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="L17">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M17">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -873,31 +880,31 @@
         <v>720</v>
       </c>
       <c r="G18" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="0"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H18" t="b">
-        <f>$C$3&gt;F18</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="I18">
-        <f t="shared" si="0"/>
-        <v>170</v>
+        <f t="shared" si="3"/>
+        <v>159</v>
       </c>
       <c r="J18" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="K18">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="L18">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="L18">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M18">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -906,31 +913,31 @@
         <v>725</v>
       </c>
       <c r="G19" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="0"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H19" t="b">
-        <f>$C$3&gt;F19</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="I19">
-        <f t="shared" si="0"/>
-        <v>170</v>
+        <f t="shared" si="3"/>
+        <v>159</v>
       </c>
       <c r="J19" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="K19">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="L19">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="L19">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M19">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -939,31 +946,31 @@
         <v>730</v>
       </c>
       <c r="G20" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="0"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H20" t="b">
-        <f>$C$3&gt;F20</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="I20">
-        <f t="shared" si="0"/>
-        <v>170</v>
+        <f t="shared" si="3"/>
+        <v>159</v>
       </c>
       <c r="J20" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="K20">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="L20">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="L20">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M20">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -972,31 +979,31 @@
         <v>735</v>
       </c>
       <c r="G21" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="0"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H21" t="b">
-        <f>$C$3&gt;F21</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="I21">
-        <f t="shared" si="0"/>
-        <v>170</v>
+        <f t="shared" si="3"/>
+        <v>159</v>
       </c>
       <c r="J21" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="K21">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="L21">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="L21">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M21">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -1005,31 +1012,31 @@
         <v>740</v>
       </c>
       <c r="G22" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="0"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H22" t="b">
-        <f>$C$3&gt;F22</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="I22">
-        <f t="shared" si="0"/>
-        <v>170</v>
+        <f t="shared" si="3"/>
+        <v>159</v>
       </c>
       <c r="J22" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="K22">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="L22">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="L22">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M22">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -1038,31 +1045,31 @@
         <v>745</v>
       </c>
       <c r="G23" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="0"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H23" t="b">
-        <f>$C$3&gt;F23</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="I23">
-        <f t="shared" si="0"/>
-        <v>170</v>
+        <f t="shared" si="3"/>
+        <v>159</v>
       </c>
       <c r="J23" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="K23">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="L23">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="L23">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -1071,32 +1078,32 @@
         <v>750</v>
       </c>
       <c r="G24" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="0"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H24" t="b">
-        <f>$C$3&gt;F24</f>
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>1</v>
       </c>
       <c r="I24">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f t="shared" si="3"/>
+        <v>159</v>
       </c>
       <c r="J24" t="b">
-        <f t="shared" si="1"/>
-        <v>1</v>
+        <f t="shared" si="4"/>
+        <v>0</v>
       </c>
       <c r="K24">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="L24">
         <f t="shared" si="2"/>
-        <v>120</v>
-      </c>
-      <c r="L24">
-        <f t="shared" si="3"/>
-        <v>0.19849537037037043</v>
+        <v>1</v>
       </c>
       <c r="M24">
-        <f t="shared" si="4"/>
-        <v>23.819444444444454</v>
+        <f t="shared" si="6"/>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="6:13" x14ac:dyDescent="0.35">
@@ -1104,32 +1111,32 @@
         <v>755</v>
       </c>
       <c r="G25" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="0"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H25" t="b">
-        <f>$C$3&gt;F25</f>
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>1</v>
       </c>
       <c r="I25">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f t="shared" si="3"/>
+        <v>159</v>
       </c>
       <c r="J25" t="b">
-        <f t="shared" si="1"/>
-        <v>1</v>
+        <f t="shared" si="4"/>
+        <v>0</v>
       </c>
       <c r="K25">
-        <f t="shared" si="2"/>
-        <v>120</v>
+        <f t="shared" si="5"/>
+        <v>0</v>
       </c>
       <c r="L25">
-        <f t="shared" si="3"/>
-        <v>0.19849537037037043</v>
+        <f>IF(AND(J25,$C$4&lt;=$C$2),(($C$1-$C$2)/($C$1-$C$4))^3,1)</f>
+        <v>1</v>
       </c>
       <c r="M25">
-        <f t="shared" si="4"/>
-        <v>23.819444444444454</v>
+        <f t="shared" si="6"/>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="6:13" x14ac:dyDescent="0.35">
@@ -1137,32 +1144,32 @@
         <v>760</v>
       </c>
       <c r="G26" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="0"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H26" t="b">
-        <f>$C$3&gt;F26</f>
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>1</v>
       </c>
       <c r="I26">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f t="shared" si="3"/>
+        <v>159</v>
       </c>
       <c r="J26" t="b">
-        <f t="shared" si="1"/>
-        <v>1</v>
+        <f t="shared" si="4"/>
+        <v>0</v>
       </c>
       <c r="K26">
-        <f t="shared" si="2"/>
-        <v>120</v>
+        <f t="shared" si="5"/>
+        <v>0</v>
       </c>
       <c r="L26">
-        <f t="shared" si="3"/>
-        <v>0.19849537037037043</v>
+        <f t="shared" ref="L26:L58" si="7">IF(AND(J26,$C$4&lt;=$C$2),(($C$1-$C$2)/($C$1-$C$4))^3,1)</f>
+        <v>1</v>
       </c>
       <c r="M26">
-        <f t="shared" si="4"/>
-        <v>23.819444444444454</v>
+        <f t="shared" si="6"/>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="6:13" x14ac:dyDescent="0.35">
@@ -1170,32 +1177,32 @@
         <v>765</v>
       </c>
       <c r="G27" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="0"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H27" t="b">
-        <f>$C$3&gt;F27</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="I27">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J27" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="K27">
-        <f t="shared" si="2"/>
-        <v>120</v>
+        <f t="shared" si="5"/>
+        <v>59</v>
       </c>
       <c r="L27">
-        <f t="shared" si="3"/>
-        <v>0.19849537037037043</v>
+        <f t="shared" si="7"/>
+        <v>1</v>
       </c>
       <c r="M27">
-        <f t="shared" si="4"/>
-        <v>23.819444444444454</v>
+        <f t="shared" si="6"/>
+        <v>59</v>
       </c>
     </row>
     <row r="28" spans="6:13" x14ac:dyDescent="0.35">
@@ -1203,32 +1210,32 @@
         <v>770</v>
       </c>
       <c r="G28" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="0"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H28" t="b">
-        <f>$C$3&gt;F28</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="I28">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J28" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="K28">
-        <f t="shared" si="2"/>
-        <v>120</v>
+        <f t="shared" si="5"/>
+        <v>59</v>
       </c>
       <c r="L28">
-        <f t="shared" si="3"/>
-        <v>0.19849537037037043</v>
+        <f t="shared" si="7"/>
+        <v>1</v>
       </c>
       <c r="M28">
-        <f t="shared" si="4"/>
-        <v>23.819444444444454</v>
+        <f t="shared" si="6"/>
+        <v>59</v>
       </c>
     </row>
     <row r="29" spans="6:13" x14ac:dyDescent="0.35">
@@ -1236,32 +1243,32 @@
         <v>775</v>
       </c>
       <c r="G29" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="0"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H29" t="b">
-        <f>$C$3&gt;F29</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="I29">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J29" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="K29">
-        <f t="shared" si="2"/>
-        <v>120</v>
+        <f t="shared" si="5"/>
+        <v>59</v>
       </c>
       <c r="L29">
-        <f t="shared" si="3"/>
-        <v>0.19849537037037043</v>
+        <f t="shared" si="7"/>
+        <v>1</v>
       </c>
       <c r="M29">
-        <f t="shared" si="4"/>
-        <v>23.819444444444454</v>
+        <f t="shared" si="6"/>
+        <v>59</v>
       </c>
     </row>
     <row r="30" spans="6:13" x14ac:dyDescent="0.35">
@@ -1269,32 +1276,32 @@
         <v>780</v>
       </c>
       <c r="G30" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="0"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H30" t="b">
-        <f>$C$3&gt;F30</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="I30">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J30" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="K30">
-        <f t="shared" si="2"/>
-        <v>120</v>
+        <f t="shared" si="5"/>
+        <v>59</v>
       </c>
       <c r="L30">
-        <f t="shared" si="3"/>
-        <v>0.19849537037037043</v>
+        <f t="shared" si="7"/>
+        <v>1</v>
       </c>
       <c r="M30">
-        <f t="shared" si="4"/>
-        <v>23.819444444444454</v>
+        <f t="shared" si="6"/>
+        <v>59</v>
       </c>
     </row>
     <row r="31" spans="6:13" x14ac:dyDescent="0.35">
@@ -1302,32 +1309,32 @@
         <v>785</v>
       </c>
       <c r="G31" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="0"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H31" t="b">
-        <f>$C$3&gt;F31</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="I31">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J31" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="K31">
-        <f t="shared" si="2"/>
-        <v>120</v>
+        <f t="shared" si="5"/>
+        <v>59</v>
       </c>
       <c r="L31">
-        <f t="shared" si="3"/>
-        <v>0.19849537037037043</v>
+        <f t="shared" si="7"/>
+        <v>1</v>
       </c>
       <c r="M31">
-        <f t="shared" si="4"/>
-        <v>23.819444444444454</v>
+        <f t="shared" si="6"/>
+        <v>59</v>
       </c>
     </row>
     <row r="32" spans="6:13" x14ac:dyDescent="0.35">
@@ -1335,32 +1342,32 @@
         <v>790</v>
       </c>
       <c r="G32" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="0"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H32" t="b">
-        <f>$C$3&gt;F32</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="I32">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J32" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="K32">
-        <f t="shared" si="2"/>
-        <v>120</v>
+        <f t="shared" si="5"/>
+        <v>59</v>
       </c>
       <c r="L32">
-        <f t="shared" si="3"/>
-        <v>0.19849537037037043</v>
+        <f t="shared" si="7"/>
+        <v>1</v>
       </c>
       <c r="M32">
-        <f t="shared" si="4"/>
-        <v>23.819444444444454</v>
+        <f t="shared" si="6"/>
+        <v>59</v>
       </c>
     </row>
     <row r="33" spans="6:13" x14ac:dyDescent="0.35">
@@ -1368,32 +1375,32 @@
         <v>795</v>
       </c>
       <c r="G33" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="0"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H33" t="b">
-        <f>$C$3&gt;F33</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="I33">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J33" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="K33">
-        <f t="shared" si="2"/>
-        <v>120</v>
+        <f t="shared" si="5"/>
+        <v>59</v>
       </c>
       <c r="L33">
-        <f t="shared" si="3"/>
-        <v>0.19849537037037043</v>
+        <f t="shared" si="7"/>
+        <v>1</v>
       </c>
       <c r="M33">
-        <f t="shared" si="4"/>
-        <v>23.819444444444454</v>
+        <f t="shared" si="6"/>
+        <v>59</v>
       </c>
     </row>
     <row r="34" spans="6:13" x14ac:dyDescent="0.35">
@@ -1401,32 +1408,32 @@
         <v>800</v>
       </c>
       <c r="G34" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="0"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H34" t="b">
-        <f>$C$3&gt;F34</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="I34">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J34" t="b">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="4"/>
+        <v>1</v>
       </c>
       <c r="K34">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <f t="shared" si="5"/>
+        <v>59</v>
       </c>
       <c r="L34">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <f t="shared" si="7"/>
+        <v>1</v>
       </c>
       <c r="M34">
-        <f t="shared" si="4"/>
-        <v>0</v>
+        <f t="shared" si="6"/>
+        <v>59</v>
       </c>
     </row>
     <row r="35" spans="6:13" x14ac:dyDescent="0.35">
@@ -1434,32 +1441,32 @@
         <v>805</v>
       </c>
       <c r="G35" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="0"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H35" t="b">
-        <f>$C$3&gt;F35</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="I35">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J35" t="b">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="4"/>
+        <v>1</v>
       </c>
       <c r="K35">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <f t="shared" si="5"/>
+        <v>59</v>
       </c>
       <c r="L35">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <f t="shared" si="7"/>
+        <v>1</v>
       </c>
       <c r="M35">
-        <f t="shared" si="4"/>
-        <v>0</v>
+        <f t="shared" si="6"/>
+        <v>59</v>
       </c>
     </row>
     <row r="36" spans="6:13" x14ac:dyDescent="0.35">
@@ -1467,32 +1474,32 @@
         <v>810</v>
       </c>
       <c r="G36" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="0"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H36" t="b">
-        <f>$C$3&gt;F36</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="I36">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J36" t="b">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="4"/>
+        <v>1</v>
       </c>
       <c r="K36">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <f t="shared" si="5"/>
+        <v>59</v>
       </c>
       <c r="L36">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <f t="shared" si="7"/>
+        <v>1</v>
       </c>
       <c r="M36">
-        <f t="shared" si="4"/>
-        <v>0</v>
+        <f t="shared" si="6"/>
+        <v>59</v>
       </c>
     </row>
     <row r="37" spans="6:13" x14ac:dyDescent="0.35">
@@ -1500,32 +1507,32 @@
         <v>815</v>
       </c>
       <c r="G37" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="0"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H37" t="b">
-        <f>$C$3&gt;F37</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="I37">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J37" t="b">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="4"/>
+        <v>1</v>
       </c>
       <c r="K37">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <f t="shared" si="5"/>
+        <v>59</v>
       </c>
       <c r="L37">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <f t="shared" si="7"/>
+        <v>1</v>
       </c>
       <c r="M37">
-        <f t="shared" si="4"/>
-        <v>0</v>
+        <f t="shared" si="6"/>
+        <v>59</v>
       </c>
     </row>
     <row r="38" spans="6:13" x14ac:dyDescent="0.35">
@@ -1533,32 +1540,32 @@
         <v>820</v>
       </c>
       <c r="G38" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="0"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H38" t="b">
-        <f>$C$3&gt;F38</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="I38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J38" t="b">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="4"/>
+        <v>1</v>
       </c>
       <c r="K38">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <f t="shared" si="5"/>
+        <v>59</v>
       </c>
       <c r="L38">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <f t="shared" si="7"/>
+        <v>1</v>
       </c>
       <c r="M38">
-        <f t="shared" si="4"/>
-        <v>0</v>
+        <f t="shared" si="6"/>
+        <v>59</v>
       </c>
     </row>
     <row r="39" spans="6:13" x14ac:dyDescent="0.35">
@@ -1566,32 +1573,32 @@
         <v>825</v>
       </c>
       <c r="G39" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="0"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H39" t="b">
-        <f>$C$3&gt;F39</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="I39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J39" t="b">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="4"/>
+        <v>1</v>
       </c>
       <c r="K39">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <f t="shared" si="5"/>
+        <v>59</v>
       </c>
       <c r="L39">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <f t="shared" si="7"/>
+        <v>1</v>
       </c>
       <c r="M39">
-        <f t="shared" si="4"/>
-        <v>0</v>
+        <f t="shared" si="6"/>
+        <v>59</v>
       </c>
     </row>
     <row r="40" spans="6:13" x14ac:dyDescent="0.35">
@@ -1599,32 +1606,32 @@
         <v>830</v>
       </c>
       <c r="G40" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" ref="G40:G58" si="8">1/COUNT($F$8:$F$58)</f>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H40" t="b">
-        <f>$C$3&gt;F40</f>
+        <f t="shared" ref="H40:H58" si="9">$C$3&gt;F40</f>
         <v>0</v>
       </c>
       <c r="I40">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J40" t="b">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="4"/>
+        <v>1</v>
       </c>
       <c r="K40">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <f t="shared" si="5"/>
+        <v>59</v>
       </c>
       <c r="L40">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <f t="shared" si="7"/>
+        <v>1</v>
       </c>
       <c r="M40">
-        <f t="shared" si="4"/>
-        <v>0</v>
+        <f t="shared" si="6"/>
+        <v>59</v>
       </c>
     </row>
     <row r="41" spans="6:13" x14ac:dyDescent="0.35">
@@ -1632,32 +1639,32 @@
         <v>835</v>
       </c>
       <c r="G41" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="8"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H41" t="b">
-        <f>$C$3&gt;F41</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="I41">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J41" t="b">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="4"/>
+        <v>1</v>
       </c>
       <c r="K41">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <f t="shared" si="5"/>
+        <v>59</v>
       </c>
       <c r="L41">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <f t="shared" si="7"/>
+        <v>1</v>
       </c>
       <c r="M41">
-        <f t="shared" si="4"/>
-        <v>0</v>
+        <f t="shared" si="6"/>
+        <v>59</v>
       </c>
     </row>
     <row r="42" spans="6:13" x14ac:dyDescent="0.35">
@@ -1665,32 +1672,32 @@
         <v>840</v>
       </c>
       <c r="G42" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="8"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H42" t="b">
-        <f>$C$3&gt;F42</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="I42">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J42" t="b">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="4"/>
+        <v>1</v>
       </c>
       <c r="K42">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <f t="shared" si="5"/>
+        <v>59</v>
       </c>
       <c r="L42">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <f t="shared" si="7"/>
+        <v>1</v>
       </c>
       <c r="M42">
-        <f t="shared" si="4"/>
-        <v>0</v>
+        <f t="shared" si="6"/>
+        <v>59</v>
       </c>
     </row>
     <row r="43" spans="6:13" x14ac:dyDescent="0.35">
@@ -1698,32 +1705,32 @@
         <v>845</v>
       </c>
       <c r="G43" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="8"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H43" t="b">
-        <f>$C$3&gt;F43</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="I43">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J43" t="b">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="4"/>
+        <v>1</v>
       </c>
       <c r="K43">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <f t="shared" si="5"/>
+        <v>59</v>
       </c>
       <c r="L43">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <f t="shared" si="7"/>
+        <v>1</v>
       </c>
       <c r="M43">
-        <f t="shared" si="4"/>
-        <v>0</v>
+        <f t="shared" si="6"/>
+        <v>59</v>
       </c>
     </row>
     <row r="44" spans="6:13" x14ac:dyDescent="0.35">
@@ -1731,32 +1738,32 @@
         <v>850</v>
       </c>
       <c r="G44" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="8"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H44" t="b">
-        <f>$C$3&gt;F44</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="I44">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J44" t="b">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="4"/>
+        <v>1</v>
       </c>
       <c r="K44">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <f t="shared" si="5"/>
+        <v>59</v>
       </c>
       <c r="L44">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <f t="shared" si="7"/>
+        <v>1</v>
       </c>
       <c r="M44">
-        <f t="shared" si="4"/>
-        <v>0</v>
+        <f t="shared" si="6"/>
+        <v>59</v>
       </c>
     </row>
     <row r="45" spans="6:13" x14ac:dyDescent="0.35">
@@ -1764,32 +1771,32 @@
         <v>855</v>
       </c>
       <c r="G45" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="8"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H45" t="b">
-        <f>$C$3&gt;F45</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="I45">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J45" t="b">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="4"/>
+        <v>1</v>
       </c>
       <c r="K45">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <f t="shared" si="5"/>
+        <v>59</v>
       </c>
       <c r="L45">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <f t="shared" si="7"/>
+        <v>1</v>
       </c>
       <c r="M45">
-        <f t="shared" si="4"/>
-        <v>0</v>
+        <f t="shared" si="6"/>
+        <v>59</v>
       </c>
     </row>
     <row r="46" spans="6:13" x14ac:dyDescent="0.35">
@@ -1797,32 +1804,32 @@
         <v>860</v>
       </c>
       <c r="G46" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="8"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H46" t="b">
-        <f>$C$3&gt;F46</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="I46">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J46" t="b">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="4"/>
+        <v>1</v>
       </c>
       <c r="K46">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <f t="shared" si="5"/>
+        <v>59</v>
       </c>
       <c r="L46">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <f t="shared" si="7"/>
+        <v>1</v>
       </c>
       <c r="M46">
-        <f t="shared" si="4"/>
-        <v>0</v>
+        <f t="shared" si="6"/>
+        <v>59</v>
       </c>
     </row>
     <row r="47" spans="6:13" x14ac:dyDescent="0.35">
@@ -1830,31 +1837,31 @@
         <v>865</v>
       </c>
       <c r="G47" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="8"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H47" t="b">
-        <f>$C$3&gt;F47</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="I47">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J47" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="K47">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="L47">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <f t="shared" si="7"/>
+        <v>1</v>
       </c>
       <c r="M47">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -1863,31 +1870,31 @@
         <v>870</v>
       </c>
       <c r="G48" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="8"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H48" t="b">
-        <f>$C$3&gt;F48</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="I48">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J48" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="K48">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="L48">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <f t="shared" si="7"/>
+        <v>1</v>
       </c>
       <c r="M48">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -1896,31 +1903,31 @@
         <v>875</v>
       </c>
       <c r="G49" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="8"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H49" t="b">
-        <f>$C$3&gt;F49</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="I49">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J49" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="K49">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="L49">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <f t="shared" si="7"/>
+        <v>1</v>
       </c>
       <c r="M49">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -1929,31 +1936,31 @@
         <v>880</v>
       </c>
       <c r="G50" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="8"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H50" t="b">
-        <f>$C$3&gt;F50</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="I50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J50" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="K50">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="L50">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <f t="shared" si="7"/>
+        <v>1</v>
       </c>
       <c r="M50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -1962,31 +1969,31 @@
         <v>885</v>
       </c>
       <c r="G51" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="8"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H51" t="b">
-        <f>$C$3&gt;F51</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="I51">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J51" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="K51">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="L51">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <f t="shared" si="7"/>
+        <v>1</v>
       </c>
       <c r="M51">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -1995,31 +2002,31 @@
         <v>890</v>
       </c>
       <c r="G52" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="8"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H52" t="b">
-        <f>$C$3&gt;F52</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="I52">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J52" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="K52">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="L52">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <f t="shared" si="7"/>
+        <v>1</v>
       </c>
       <c r="M52">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -2028,31 +2035,31 @@
         <v>895</v>
       </c>
       <c r="G53" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="8"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H53" t="b">
-        <f>$C$3&gt;F53</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="I53">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J53" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="K53">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="L53">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <f t="shared" si="7"/>
+        <v>1</v>
       </c>
       <c r="M53">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -2061,31 +2068,31 @@
         <v>900</v>
       </c>
       <c r="G54" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="8"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H54" t="b">
-        <f>$C$3&gt;F54</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="I54">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J54" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="K54">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="L54">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <f t="shared" si="7"/>
+        <v>1</v>
       </c>
       <c r="M54">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -2094,31 +2101,31 @@
         <v>905</v>
       </c>
       <c r="G55" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="8"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H55" t="b">
-        <f>$C$3&gt;F55</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="I55">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J55" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="K55">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="L55">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <f t="shared" si="7"/>
+        <v>1</v>
       </c>
       <c r="M55">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -2127,31 +2134,31 @@
         <v>910</v>
       </c>
       <c r="G56" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="8"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H56" t="b">
-        <f>$C$3&gt;F56</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="I56">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J56" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="K56">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="L56">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <f t="shared" si="7"/>
+        <v>1</v>
       </c>
       <c r="M56">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -2160,31 +2167,31 @@
         <v>915</v>
       </c>
       <c r="G57" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="8"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H57" t="b">
-        <f>$C$3&gt;F57</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="I57">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J57" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="K57">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="L57">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <f t="shared" si="7"/>
+        <v>1</v>
       </c>
       <c r="M57">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -2193,46 +2200,55 @@
         <v>920</v>
       </c>
       <c r="G58" s="1">
-        <f>1/COUNT($F$8:$F$58)</f>
+        <f t="shared" si="8"/>
         <v>1.9607843137254902E-2</v>
       </c>
       <c r="H58" t="b">
-        <f>$C$3&gt;F58</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="I58">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J58" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="K58">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="L58">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <f t="shared" si="7"/>
+        <v>1</v>
       </c>
       <c r="M58">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
     <row r="59" spans="6:14" x14ac:dyDescent="0.35">
       <c r="I59">
         <f>SUM(I8:I58)</f>
-        <v>2720</v>
+        <v>3021</v>
       </c>
       <c r="M59">
         <f>SUM(M8:M58)</f>
-        <v>238.19444444444454</v>
+        <v>1180</v>
       </c>
       <c r="N59">
         <f>SUM(I59,M59)</f>
-        <v>2958.1944444444443</v>
+        <v>4201</v>
+      </c>
+    </row>
+    <row r="62" spans="6:14" x14ac:dyDescent="0.35">
+      <c r="M62" t="s">
+        <v>14</v>
+      </c>
+      <c r="N62">
+        <f>N59/4301</f>
+        <v>0.97674959311787957</v>
       </c>
     </row>
   </sheetData>

</xml_diff>